<commit_message>
add docker to project
</commit_message>
<xml_diff>
--- a/data/Notes.xlsx
+++ b/data/Notes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,12 +461,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>note-1</t>
+          <t>note-3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-16T16:11:21</t>
+          <t>2026-04-16T16:36:31</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -481,141 +481,25 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Profile change request submitted by user.</t>
+          <t>New dependant added by user. Please review.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>RESOLVED</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>teri@haycarb.com</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Updated in SHE by admin.</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>CHANGE</t>
+          <t>DEPENDANT_ADD</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>she-10</t>
+          <t>she-12</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
-        <is>
-          <t>{"name": "W L A M SIRIWARDANa"}</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>note-2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-04-16T16:17:39</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>ams@haycarb.com</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>920272363V</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Profile change request submitted by user.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>RESOLVED</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>teri@haycarb.com</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Updated in SHE by admin.</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>CHANGE</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>she-10</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>{"name": "W L A M SIRIWARDANE"}</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>note-3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-04-16T16:36:31</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>ams@haycarb.com</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>920272363V</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>New dependant added by user. Please review.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>DEPENDANT_ADD</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>she-12</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
         <is>
           <t>{"name": "Akash", "nic": "920272363V", "relation": "Son", "dob": "2024-06-16", "gender": "Male"}</t>
         </is>

</xml_diff>